<commit_message>
feat: weight lookup output (ID + weight columns) with id_column config
Key changes:
- Output file now produces clean weight lookup (respondent ID in col A,
  weight columns in subsequent columns) instead of full dataset dump
- Add id_column config setting (auto-detects first column if not set)
- tryCatch handlers pass through TRS refusals via turas_refusal condition
- Fix reference-level verbose message (only fires for actual reference)
- Regenerate config template with id_column setting
- Update all docs: CODE_INVENTORY, CONFIG_EXAMPLE, TEMPLATE_REFERENCE,
  TECHNICAL_DOCS, USER_MANUAL, README
- Update output tests for new signature and add id_column validation test
- Successfully ran CCS-W4 demo: 160 respondents, 92% efficiency, GOOD

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/modules/weighting/docs/templates/Weight_Config_Template.xlsx
+++ b/modules/weighting/docs/templates/Weight_Config_Template.xlsx
@@ -6,7 +6,7 @@
     <workbookView xWindow="0" yWindow="0" windowWidth="13125" windowHeight="6105" firstSheet="0" activeTab="0"/>
   </bookViews>
   <sheets>
-    <sheet name="Settings" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="General" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Weight_Specifications" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="Design_Targets" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="Rim_Targets" sheetId="4" state="visible" r:id="rId4"/>
@@ -18,7 +18,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="138" uniqueCount="138">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="136" uniqueCount="136">
   <si>
     <t xml:space="preserve">TURAS Weighting Module - Configuration</t>
   </si>
@@ -83,10 +83,22 @@
     <t xml:space="preserve">Relative or absolute file path, e.g. 'data/survey.csv'</t>
   </si>
   <si>
+    <t xml:space="preserve">id_column</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ResponseID</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Name of the respondent ID column in the data file. Used to produce the weight lookup file (ID + Weight columns only)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Column name from your data, e.g. 'ResponseID', 'resp_id', 'ID'</t>
+  </si>
+  <si>
     <t xml:space="preserve">output_file</t>
   </si>
   <si>
-    <t xml:space="preserve">Path for the weighted output file (CSV or Excel). If blank, auto-generated from data_file</t>
+    <t xml:space="preserve">Path for the weight lookup file (ID + weight columns). If blank, auto-generated from data_file</t>
   </si>
   <si>
     <t xml:space="preserve">File path with .csv or .xlsx extension</t>
@@ -347,31 +359,13 @@
     <t xml:space="preserve">Define joint target percentages for cross-classified cells. All cells for each weight must sum to 100%.</t>
   </si>
   <si>
-    <t xml:space="preserve">Variable_1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Value_1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Variable_2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Value_2</t>
-  </si>
-  <si>
     <t xml:space="preserve">[REQUIRED] Must match a weight_name from Weight_Specifications with method=cell.</t>
   </si>
   <si>
-    <t xml:space="preserve">[REQUIRED] First interlocking variable column name in your data.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">[REQUIRED] Category value for the first variable (must match data values exactly).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">[REQUIRED] Second interlocking variable column name in your data.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">[REQUIRED] Category value for the second variable (must match data values exactly).</t>
+    <t xml:space="preserve">[REQUIRED] EXAMPLE column — rename to your first interlocking variable. Values must match data exactly.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">[REQUIRED] EXAMPLE column — rename to your second interlocking variable. Values must match data exactly.</t>
   </si>
   <si>
     <t xml:space="preserve">[REQUIRED] Target population percentage for this cell combination. All cells for a weight must sum to 100.</t>
@@ -1043,24 +1037,24 @@
         <v>21</v>
       </c>
       <c r="B9" s="11" t="s">
-        <v>14</v>
+        <v>22</v>
       </c>
       <c r="C9" s="16" t="s">
         <v>4</v>
       </c>
       <c r="D9" s="13" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="E9" s="14" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="15" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B10" s="11" t="s">
-        <v>25</v>
+        <v>14</v>
       </c>
       <c r="C10" s="16" t="s">
         <v>4</v>
@@ -1077,77 +1071,77 @@
         <v>28</v>
       </c>
       <c r="B11" s="11" t="s">
-        <v>14</v>
+        <v>29</v>
       </c>
       <c r="C11" s="16" t="s">
         <v>4</v>
       </c>
       <c r="D11" s="13" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="E11" s="14" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="15" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B12" s="11" t="s">
-        <v>25</v>
+        <v>14</v>
       </c>
       <c r="C12" s="16" t="s">
         <v>4</v>
       </c>
       <c r="D12" s="13" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="E12" s="14" t="s">
-        <v>27</v>
+        <v>34</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="15" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="B13" s="11" t="s">
-        <v>14</v>
+        <v>29</v>
       </c>
       <c r="C13" s="16" t="s">
         <v>4</v>
       </c>
       <c r="D13" s="13" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="E13" s="14" t="s">
-        <v>35</v>
+        <v>31</v>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="9" t="s">
-        <v>36</v>
-      </c>
-      <c r="B14" s="9"/>
-      <c r="C14" s="9"/>
-      <c r="D14" s="9"/>
-      <c r="E14" s="9"/>
+      <c r="A14" s="15" t="s">
+        <v>37</v>
+      </c>
+      <c r="B14" s="11" t="s">
+        <v>14</v>
+      </c>
+      <c r="C14" s="16" t="s">
+        <v>4</v>
+      </c>
+      <c r="D14" s="13" t="s">
+        <v>38</v>
+      </c>
+      <c r="E14" s="14" t="s">
+        <v>39</v>
+      </c>
     </row>
     <row r="15">
-      <c r="A15" s="15" t="s">
-        <v>37</v>
-      </c>
-      <c r="B15" s="11" t="s">
-        <v>38</v>
-      </c>
-      <c r="C15" s="16" t="s">
-        <v>4</v>
-      </c>
-      <c r="D15" s="13" t="s">
-        <v>39</v>
-      </c>
-      <c r="E15" s="14" t="s">
+      <c r="A15" s="9" t="s">
         <v>40</v>
       </c>
+      <c r="B15" s="9"/>
+      <c r="C15" s="9"/>
+      <c r="D15" s="9"/>
+      <c r="E15" s="9"/>
     </row>
     <row r="16">
       <c r="A16" s="15" t="s">
@@ -1171,21 +1165,21 @@
         <v>45</v>
       </c>
       <c r="B17" s="11" t="s">
-        <v>14</v>
+        <v>46</v>
       </c>
       <c r="C17" s="16" t="s">
         <v>4</v>
       </c>
       <c r="D17" s="13" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="E17" s="14" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="15" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="B18" s="11" t="s">
         <v>14</v>
@@ -1194,15 +1188,15 @@
         <v>4</v>
       </c>
       <c r="D18" s="13" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="E18" s="14" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="15" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="B19" s="11" t="s">
         <v>14</v>
@@ -1211,10 +1205,27 @@
         <v>4</v>
       </c>
       <c r="D19" s="13" t="s">
+        <v>53</v>
+      </c>
+      <c r="E19" s="14" t="s">
         <v>51</v>
       </c>
-      <c r="E19" s="14" t="s">
-        <v>52</v>
+    </row>
+    <row r="20">
+      <c r="A20" s="15" t="s">
+        <v>54</v>
+      </c>
+      <c r="B20" s="11" t="s">
+        <v>14</v>
+      </c>
+      <c r="C20" s="16" t="s">
+        <v>4</v>
+      </c>
+      <c r="D20" s="13" t="s">
+        <v>55</v>
+      </c>
+      <c r="E20" s="14" t="s">
+        <v>56</v>
       </c>
     </row>
   </sheetData>
@@ -1222,7 +1233,7 @@
     <mergeCell ref="A1:E1"/>
     <mergeCell ref="A2:E2"/>
     <mergeCell ref="A6:E6"/>
-    <mergeCell ref="A14:E14"/>
+    <mergeCell ref="A15:E15"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
@@ -1233,13 +1244,13 @@
           <x14:formula1>
             <xm:f>"Y,N"</xm:f>
           </x14:formula1>
-          <xm:sqref>B10:B10</xm:sqref>
+          <xm:sqref>B11:B11</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1">
           <x14:formula1>
             <xm:f>"Y,N"</xm:f>
           </x14:formula1>
-          <xm:sqref>B12:B12</xm:sqref>
+          <xm:sqref>B13:B13</xm:sqref>
         </x14:dataValidation>
       </x14:dataValidations>
     </ext>
@@ -1262,69 +1273,69 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="s">
-        <v>54</v>
+        <v>58</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="8" t="s">
-        <v>55</v>
+        <v>59</v>
       </c>
       <c r="B3" s="8" t="s">
-        <v>56</v>
+        <v>60</v>
       </c>
       <c r="C3" s="8" t="s">
-        <v>57</v>
+        <v>61</v>
       </c>
       <c r="D3" s="8" t="s">
-        <v>58</v>
+        <v>62</v>
       </c>
       <c r="E3" s="8" t="s">
-        <v>59</v>
+        <v>63</v>
       </c>
       <c r="F3" s="8" t="s">
-        <v>60</v>
+        <v>64</v>
       </c>
     </row>
     <row r="4" ht="45" customHeight="1">
       <c r="A4" s="13" t="s">
-        <v>61</v>
+        <v>65</v>
       </c>
       <c r="B4" s="13" t="s">
-        <v>62</v>
+        <v>66</v>
       </c>
       <c r="C4" s="13" t="s">
-        <v>63</v>
+        <v>67</v>
       </c>
       <c r="D4" s="13" t="s">
-        <v>64</v>
+        <v>68</v>
       </c>
       <c r="E4" s="13" t="s">
-        <v>65</v>
+        <v>69</v>
       </c>
       <c r="F4" s="13" t="s">
-        <v>66</v>
+        <v>70</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="17" t="s">
-        <v>67</v>
+        <v>71</v>
       </c>
       <c r="B5" s="17" t="s">
-        <v>68</v>
+        <v>72</v>
       </c>
       <c r="C5" s="17" t="s">
-        <v>69</v>
+        <v>73</v>
       </c>
       <c r="D5" s="17" t="s">
-        <v>70</v>
+        <v>74</v>
       </c>
       <c r="E5" s="17" t="s">
-        <v>71</v>
+        <v>75</v>
       </c>
       <c r="F5" s="17" t="n">
         <v>5</v>
@@ -1332,16 +1343,16 @@
     </row>
     <row r="6">
       <c r="A6" s="17" t="s">
-        <v>72</v>
+        <v>76</v>
       </c>
       <c r="B6" s="17" t="s">
-        <v>73</v>
+        <v>77</v>
       </c>
       <c r="C6" s="17" t="s">
-        <v>74</v>
+        <v>78</v>
       </c>
       <c r="D6" s="17" t="s">
-        <v>25</v>
+        <v>29</v>
       </c>
       <c r="E6" s="17" t="s">
         <v>14</v>
@@ -1352,19 +1363,19 @@
     </row>
     <row r="7">
       <c r="A7" s="17" t="s">
-        <v>75</v>
+        <v>79</v>
       </c>
       <c r="B7" s="17" t="s">
-        <v>76</v>
+        <v>80</v>
       </c>
       <c r="C7" s="17" t="s">
-        <v>77</v>
+        <v>81</v>
       </c>
       <c r="D7" s="17" t="s">
-        <v>70</v>
+        <v>74</v>
       </c>
       <c r="E7" s="17" t="s">
-        <v>78</v>
+        <v>82</v>
       </c>
       <c r="F7" s="17" t="n">
         <v>95</v>
@@ -1577,51 +1588,51 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="s">
-        <v>80</v>
+        <v>84</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="8" t="s">
-        <v>55</v>
+        <v>59</v>
       </c>
       <c r="B3" s="8" t="s">
-        <v>81</v>
+        <v>85</v>
       </c>
       <c r="C3" s="8" t="s">
-        <v>82</v>
+        <v>86</v>
       </c>
       <c r="D3" s="8" t="s">
-        <v>83</v>
+        <v>87</v>
       </c>
     </row>
     <row r="4" ht="45" customHeight="1">
       <c r="A4" s="13" t="s">
-        <v>84</v>
+        <v>88</v>
       </c>
       <c r="B4" s="13" t="s">
-        <v>85</v>
+        <v>89</v>
       </c>
       <c r="C4" s="13" t="s">
-        <v>86</v>
+        <v>90</v>
       </c>
       <c r="D4" s="13" t="s">
-        <v>87</v>
+        <v>91</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="17" t="s">
-        <v>72</v>
+        <v>76</v>
       </c>
       <c r="B5" s="17" t="s">
-        <v>88</v>
+        <v>92</v>
       </c>
       <c r="C5" s="17" t="s">
-        <v>89</v>
+        <v>93</v>
       </c>
       <c r="D5" s="17" t="n">
         <v>45000</v>
@@ -1629,13 +1640,13 @@
     </row>
     <row r="6">
       <c r="A6" s="17" t="s">
-        <v>72</v>
+        <v>76</v>
       </c>
       <c r="B6" s="17" t="s">
-        <v>88</v>
+        <v>92</v>
       </c>
       <c r="C6" s="17" t="s">
-        <v>90</v>
+        <v>94</v>
       </c>
       <c r="D6" s="17" t="n">
         <v>55000</v>
@@ -1964,51 +1975,51 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>91</v>
+        <v>95</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="s">
-        <v>92</v>
+        <v>96</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="8" t="s">
-        <v>55</v>
+        <v>59</v>
       </c>
       <c r="B3" s="8" t="s">
-        <v>93</v>
+        <v>97</v>
       </c>
       <c r="C3" s="8" t="s">
-        <v>94</v>
+        <v>98</v>
       </c>
       <c r="D3" s="8" t="s">
-        <v>95</v>
+        <v>99</v>
       </c>
     </row>
     <row r="4" ht="45" customHeight="1">
       <c r="A4" s="13" t="s">
-        <v>96</v>
+        <v>100</v>
       </c>
       <c r="B4" s="13" t="s">
-        <v>97</v>
+        <v>101</v>
       </c>
       <c r="C4" s="13" t="s">
-        <v>98</v>
+        <v>102</v>
       </c>
       <c r="D4" s="13" t="s">
-        <v>99</v>
+        <v>103</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="17" t="s">
-        <v>67</v>
+        <v>71</v>
       </c>
       <c r="B5" s="17" t="s">
-        <v>100</v>
+        <v>104</v>
       </c>
       <c r="C5" s="17" t="s">
-        <v>101</v>
+        <v>105</v>
       </c>
       <c r="D5" s="17" t="n">
         <v>48.5</v>
@@ -2016,13 +2027,13 @@
     </row>
     <row r="6">
       <c r="A6" s="17" t="s">
-        <v>67</v>
+        <v>71</v>
       </c>
       <c r="B6" s="17" t="s">
-        <v>100</v>
+        <v>104</v>
       </c>
       <c r="C6" s="17" t="s">
-        <v>102</v>
+        <v>106</v>
       </c>
       <c r="D6" s="17" t="n">
         <v>51.5</v>
@@ -2030,13 +2041,13 @@
     </row>
     <row r="7">
       <c r="A7" s="17" t="s">
-        <v>67</v>
+        <v>71</v>
       </c>
       <c r="B7" s="17" t="s">
-        <v>103</v>
+        <v>107</v>
       </c>
       <c r="C7" s="17" t="s">
-        <v>104</v>
+        <v>108</v>
       </c>
       <c r="D7" s="17" t="n">
         <v>30</v>
@@ -2044,13 +2055,13 @@
     </row>
     <row r="8">
       <c r="A8" s="17" t="s">
-        <v>67</v>
+        <v>71</v>
       </c>
       <c r="B8" s="17" t="s">
-        <v>103</v>
+        <v>107</v>
       </c>
       <c r="C8" s="17" t="s">
-        <v>105</v>
+        <v>109</v>
       </c>
       <c r="D8" s="17" t="n">
         <v>35</v>
@@ -2058,13 +2069,13 @@
     </row>
     <row r="9">
       <c r="A9" s="17" t="s">
-        <v>67</v>
+        <v>71</v>
       </c>
       <c r="B9" s="17" t="s">
-        <v>103</v>
+        <v>107</v>
       </c>
       <c r="C9" s="17" t="s">
-        <v>106</v>
+        <v>110</v>
       </c>
       <c r="D9" s="17" t="n">
         <v>35</v>
@@ -2694,39 +2705,31 @@
     <col min="1" max="1" width="25.71" hidden="0" customWidth="1"/>
     <col min="2" max="2" width="20.71" hidden="0" customWidth="1"/>
     <col min="3" max="3" width="20.71" hidden="0" customWidth="1"/>
-    <col min="4" max="4" width="20.71" hidden="0" customWidth="1"/>
-    <col min="5" max="5" width="20.71" hidden="0" customWidth="1"/>
-    <col min="6" max="6" width="18.71" hidden="0" customWidth="1"/>
+    <col min="4" max="4" width="18.71" hidden="0" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>107</v>
+        <v>111</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="s">
-        <v>108</v>
+        <v>112</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="8" t="s">
-        <v>55</v>
+        <v>59</v>
       </c>
       <c r="B3" s="8" t="s">
-        <v>109</v>
+        <v>104</v>
       </c>
       <c r="C3" s="8" t="s">
-        <v>110</v>
+        <v>107</v>
       </c>
       <c r="D3" s="8" t="s">
-        <v>111</v>
-      </c>
-      <c r="E3" s="8" t="s">
-        <v>112</v>
-      </c>
-      <c r="F3" s="8" t="s">
-        <v>95</v>
+        <v>99</v>
       </c>
     </row>
     <row r="4" ht="45" customHeight="1">
@@ -2742,70 +2745,46 @@
       <c r="D4" s="13" t="s">
         <v>116</v>
       </c>
-      <c r="E4" s="13" t="s">
-        <v>117</v>
-      </c>
-      <c r="F4" s="13" t="s">
-        <v>118</v>
-      </c>
     </row>
     <row r="5">
       <c r="A5" s="17" t="s">
-        <v>75</v>
+        <v>79</v>
       </c>
       <c r="B5" s="17" t="s">
-        <v>100</v>
+        <v>105</v>
       </c>
       <c r="C5" s="17" t="s">
-        <v>101</v>
-      </c>
-      <c r="D5" s="17" t="s">
-        <v>103</v>
-      </c>
-      <c r="E5" s="17" t="s">
-        <v>104</v>
-      </c>
-      <c r="F5" s="17" t="n">
+        <v>108</v>
+      </c>
+      <c r="D5" s="17" t="n">
         <v>15</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="17" t="s">
-        <v>75</v>
+        <v>79</v>
       </c>
       <c r="B6" s="17" t="s">
-        <v>100</v>
+        <v>105</v>
       </c>
       <c r="C6" s="17" t="s">
-        <v>101</v>
-      </c>
-      <c r="D6" s="17" t="s">
-        <v>103</v>
-      </c>
-      <c r="E6" s="17" t="s">
-        <v>105</v>
-      </c>
-      <c r="F6" s="17" t="n">
+        <v>109</v>
+      </c>
+      <c r="D6" s="17" t="n">
         <v>17</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="17" t="s">
-        <v>75</v>
+        <v>79</v>
       </c>
       <c r="B7" s="17" t="s">
-        <v>100</v>
+        <v>105</v>
       </c>
       <c r="C7" s="17" t="s">
-        <v>101</v>
-      </c>
-      <c r="D7" s="17" t="s">
-        <v>103</v>
-      </c>
-      <c r="E7" s="17" t="s">
-        <v>106</v>
-      </c>
-      <c r="F7" s="17" t="n">
+        <v>110</v>
+      </c>
+      <c r="D7" s="17" t="n">
         <v>16</v>
       </c>
     </row>
@@ -2814,408 +2793,308 @@
       <c r="B8" s="11"/>
       <c r="C8" s="11"/>
       <c r="D8" s="11"/>
-      <c r="E8" s="11"/>
-      <c r="F8" s="11"/>
     </row>
     <row r="9">
       <c r="A9" s="11"/>
       <c r="B9" s="11"/>
       <c r="C9" s="11"/>
       <c r="D9" s="11"/>
-      <c r="E9" s="11"/>
-      <c r="F9" s="11"/>
     </row>
     <row r="10">
       <c r="A10" s="11"/>
       <c r="B10" s="11"/>
       <c r="C10" s="11"/>
       <c r="D10" s="11"/>
-      <c r="E10" s="11"/>
-      <c r="F10" s="11"/>
     </row>
     <row r="11">
       <c r="A11" s="11"/>
       <c r="B11" s="11"/>
       <c r="C11" s="11"/>
       <c r="D11" s="11"/>
-      <c r="E11" s="11"/>
-      <c r="F11" s="11"/>
     </row>
     <row r="12">
       <c r="A12" s="11"/>
       <c r="B12" s="11"/>
       <c r="C12" s="11"/>
       <c r="D12" s="11"/>
-      <c r="E12" s="11"/>
-      <c r="F12" s="11"/>
     </row>
     <row r="13">
       <c r="A13" s="11"/>
       <c r="B13" s="11"/>
       <c r="C13" s="11"/>
       <c r="D13" s="11"/>
-      <c r="E13" s="11"/>
-      <c r="F13" s="11"/>
     </row>
     <row r="14">
       <c r="A14" s="11"/>
       <c r="B14" s="11"/>
       <c r="C14" s="11"/>
       <c r="D14" s="11"/>
-      <c r="E14" s="11"/>
-      <c r="F14" s="11"/>
     </row>
     <row r="15">
       <c r="A15" s="11"/>
       <c r="B15" s="11"/>
       <c r="C15" s="11"/>
       <c r="D15" s="11"/>
-      <c r="E15" s="11"/>
-      <c r="F15" s="11"/>
     </row>
     <row r="16">
       <c r="A16" s="11"/>
       <c r="B16" s="11"/>
       <c r="C16" s="11"/>
       <c r="D16" s="11"/>
-      <c r="E16" s="11"/>
-      <c r="F16" s="11"/>
     </row>
     <row r="17">
       <c r="A17" s="11"/>
       <c r="B17" s="11"/>
       <c r="C17" s="11"/>
       <c r="D17" s="11"/>
-      <c r="E17" s="11"/>
-      <c r="F17" s="11"/>
     </row>
     <row r="18">
       <c r="A18" s="11"/>
       <c r="B18" s="11"/>
       <c r="C18" s="11"/>
       <c r="D18" s="11"/>
-      <c r="E18" s="11"/>
-      <c r="F18" s="11"/>
     </row>
     <row r="19">
       <c r="A19" s="11"/>
       <c r="B19" s="11"/>
       <c r="C19" s="11"/>
       <c r="D19" s="11"/>
-      <c r="E19" s="11"/>
-      <c r="F19" s="11"/>
     </row>
     <row r="20">
       <c r="A20" s="11"/>
       <c r="B20" s="11"/>
       <c r="C20" s="11"/>
       <c r="D20" s="11"/>
-      <c r="E20" s="11"/>
-      <c r="F20" s="11"/>
     </row>
     <row r="21">
       <c r="A21" s="11"/>
       <c r="B21" s="11"/>
       <c r="C21" s="11"/>
       <c r="D21" s="11"/>
-      <c r="E21" s="11"/>
-      <c r="F21" s="11"/>
     </row>
     <row r="22">
       <c r="A22" s="11"/>
       <c r="B22" s="11"/>
       <c r="C22" s="11"/>
       <c r="D22" s="11"/>
-      <c r="E22" s="11"/>
-      <c r="F22" s="11"/>
     </row>
     <row r="23">
       <c r="A23" s="11"/>
       <c r="B23" s="11"/>
       <c r="C23" s="11"/>
       <c r="D23" s="11"/>
-      <c r="E23" s="11"/>
-      <c r="F23" s="11"/>
     </row>
     <row r="24">
       <c r="A24" s="11"/>
       <c r="B24" s="11"/>
       <c r="C24" s="11"/>
       <c r="D24" s="11"/>
-      <c r="E24" s="11"/>
-      <c r="F24" s="11"/>
     </row>
     <row r="25">
       <c r="A25" s="11"/>
       <c r="B25" s="11"/>
       <c r="C25" s="11"/>
       <c r="D25" s="11"/>
-      <c r="E25" s="11"/>
-      <c r="F25" s="11"/>
     </row>
     <row r="26">
       <c r="A26" s="11"/>
       <c r="B26" s="11"/>
       <c r="C26" s="11"/>
       <c r="D26" s="11"/>
-      <c r="E26" s="11"/>
-      <c r="F26" s="11"/>
     </row>
     <row r="27">
       <c r="A27" s="11"/>
       <c r="B27" s="11"/>
       <c r="C27" s="11"/>
       <c r="D27" s="11"/>
-      <c r="E27" s="11"/>
-      <c r="F27" s="11"/>
     </row>
     <row r="28">
       <c r="A28" s="11"/>
       <c r="B28" s="11"/>
       <c r="C28" s="11"/>
       <c r="D28" s="11"/>
-      <c r="E28" s="11"/>
-      <c r="F28" s="11"/>
     </row>
     <row r="29">
       <c r="A29" s="11"/>
       <c r="B29" s="11"/>
       <c r="C29" s="11"/>
       <c r="D29" s="11"/>
-      <c r="E29" s="11"/>
-      <c r="F29" s="11"/>
     </row>
     <row r="30">
       <c r="A30" s="11"/>
       <c r="B30" s="11"/>
       <c r="C30" s="11"/>
       <c r="D30" s="11"/>
-      <c r="E30" s="11"/>
-      <c r="F30" s="11"/>
     </row>
     <row r="31">
       <c r="A31" s="11"/>
       <c r="B31" s="11"/>
       <c r="C31" s="11"/>
       <c r="D31" s="11"/>
-      <c r="E31" s="11"/>
-      <c r="F31" s="11"/>
     </row>
     <row r="32">
       <c r="A32" s="11"/>
       <c r="B32" s="11"/>
       <c r="C32" s="11"/>
       <c r="D32" s="11"/>
-      <c r="E32" s="11"/>
-      <c r="F32" s="11"/>
     </row>
     <row r="33">
       <c r="A33" s="11"/>
       <c r="B33" s="11"/>
       <c r="C33" s="11"/>
       <c r="D33" s="11"/>
-      <c r="E33" s="11"/>
-      <c r="F33" s="11"/>
     </row>
     <row r="34">
       <c r="A34" s="11"/>
       <c r="B34" s="11"/>
       <c r="C34" s="11"/>
       <c r="D34" s="11"/>
-      <c r="E34" s="11"/>
-      <c r="F34" s="11"/>
     </row>
     <row r="35">
       <c r="A35" s="11"/>
       <c r="B35" s="11"/>
       <c r="C35" s="11"/>
       <c r="D35" s="11"/>
-      <c r="E35" s="11"/>
-      <c r="F35" s="11"/>
     </row>
     <row r="36">
       <c r="A36" s="11"/>
       <c r="B36" s="11"/>
       <c r="C36" s="11"/>
       <c r="D36" s="11"/>
-      <c r="E36" s="11"/>
-      <c r="F36" s="11"/>
     </row>
     <row r="37">
       <c r="A37" s="11"/>
       <c r="B37" s="11"/>
       <c r="C37" s="11"/>
       <c r="D37" s="11"/>
-      <c r="E37" s="11"/>
-      <c r="F37" s="11"/>
     </row>
     <row r="38">
       <c r="A38" s="11"/>
       <c r="B38" s="11"/>
       <c r="C38" s="11"/>
       <c r="D38" s="11"/>
-      <c r="E38" s="11"/>
-      <c r="F38" s="11"/>
     </row>
     <row r="39">
       <c r="A39" s="11"/>
       <c r="B39" s="11"/>
       <c r="C39" s="11"/>
       <c r="D39" s="11"/>
-      <c r="E39" s="11"/>
-      <c r="F39" s="11"/>
     </row>
     <row r="40">
       <c r="A40" s="11"/>
       <c r="B40" s="11"/>
       <c r="C40" s="11"/>
       <c r="D40" s="11"/>
-      <c r="E40" s="11"/>
-      <c r="F40" s="11"/>
     </row>
     <row r="41">
       <c r="A41" s="11"/>
       <c r="B41" s="11"/>
       <c r="C41" s="11"/>
       <c r="D41" s="11"/>
-      <c r="E41" s="11"/>
-      <c r="F41" s="11"/>
     </row>
     <row r="42">
       <c r="A42" s="11"/>
       <c r="B42" s="11"/>
       <c r="C42" s="11"/>
       <c r="D42" s="11"/>
-      <c r="E42" s="11"/>
-      <c r="F42" s="11"/>
     </row>
     <row r="43">
       <c r="A43" s="11"/>
       <c r="B43" s="11"/>
       <c r="C43" s="11"/>
       <c r="D43" s="11"/>
-      <c r="E43" s="11"/>
-      <c r="F43" s="11"/>
     </row>
     <row r="44">
       <c r="A44" s="11"/>
       <c r="B44" s="11"/>
       <c r="C44" s="11"/>
       <c r="D44" s="11"/>
-      <c r="E44" s="11"/>
-      <c r="F44" s="11"/>
     </row>
     <row r="45">
       <c r="A45" s="11"/>
       <c r="B45" s="11"/>
       <c r="C45" s="11"/>
       <c r="D45" s="11"/>
-      <c r="E45" s="11"/>
-      <c r="F45" s="11"/>
     </row>
     <row r="46">
       <c r="A46" s="11"/>
       <c r="B46" s="11"/>
       <c r="C46" s="11"/>
       <c r="D46" s="11"/>
-      <c r="E46" s="11"/>
-      <c r="F46" s="11"/>
     </row>
     <row r="47">
       <c r="A47" s="11"/>
       <c r="B47" s="11"/>
       <c r="C47" s="11"/>
       <c r="D47" s="11"/>
-      <c r="E47" s="11"/>
-      <c r="F47" s="11"/>
     </row>
     <row r="48">
       <c r="A48" s="11"/>
       <c r="B48" s="11"/>
       <c r="C48" s="11"/>
       <c r="D48" s="11"/>
-      <c r="E48" s="11"/>
-      <c r="F48" s="11"/>
     </row>
     <row r="49">
       <c r="A49" s="11"/>
       <c r="B49" s="11"/>
       <c r="C49" s="11"/>
       <c r="D49" s="11"/>
-      <c r="E49" s="11"/>
-      <c r="F49" s="11"/>
     </row>
     <row r="50">
       <c r="A50" s="11"/>
       <c r="B50" s="11"/>
       <c r="C50" s="11"/>
       <c r="D50" s="11"/>
-      <c r="E50" s="11"/>
-      <c r="F50" s="11"/>
     </row>
     <row r="51">
       <c r="A51" s="11"/>
       <c r="B51" s="11"/>
       <c r="C51" s="11"/>
       <c r="D51" s="11"/>
-      <c r="E51" s="11"/>
-      <c r="F51" s="11"/>
     </row>
     <row r="52">
       <c r="A52" s="11"/>
       <c r="B52" s="11"/>
       <c r="C52" s="11"/>
       <c r="D52" s="11"/>
-      <c r="E52" s="11"/>
-      <c r="F52" s="11"/>
     </row>
     <row r="53">
       <c r="A53" s="11"/>
       <c r="B53" s="11"/>
       <c r="C53" s="11"/>
       <c r="D53" s="11"/>
-      <c r="E53" s="11"/>
-      <c r="F53" s="11"/>
     </row>
     <row r="54">
       <c r="A54" s="11"/>
       <c r="B54" s="11"/>
       <c r="C54" s="11"/>
       <c r="D54" s="11"/>
-      <c r="E54" s="11"/>
-      <c r="F54" s="11"/>
     </row>
     <row r="55">
       <c r="A55" s="11"/>
       <c r="B55" s="11"/>
       <c r="C55" s="11"/>
       <c r="D55" s="11"/>
-      <c r="E55" s="11"/>
-      <c r="F55" s="11"/>
     </row>
     <row r="56">
       <c r="A56" s="11"/>
       <c r="B56" s="11"/>
       <c r="C56" s="11"/>
       <c r="D56" s="11"/>
-      <c r="E56" s="11"/>
-      <c r="F56" s="11"/>
     </row>
     <row r="57">
       <c r="A57" s="11"/>
       <c r="B57" s="11"/>
       <c r="C57" s="11"/>
       <c r="D57" s="11"/>
-      <c r="E57" s="11"/>
-      <c r="F57" s="11"/>
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="A1:F1"/>
-    <mergeCell ref="A2:F2"/>
+    <mergeCell ref="A1:D1"/>
+    <mergeCell ref="A2:D2"/>
   </mergeCells>
   <dataValidations count="1">
-    <dataValidation type="decimal" operator="between" allowBlank="0" showInputMessage="1" showErrorMessage="1" sqref="F5:F57">
+    <dataValidation type="decimal" operator="between" allowBlank="0" showInputMessage="1" showErrorMessage="1" sqref="D5:D57">
       <formula1>0</formula1>
       <formula2>100</formula2>
     </dataValidation>
@@ -3238,45 +3117,45 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="8" t="s">
-        <v>55</v>
+        <v>59</v>
       </c>
       <c r="B3" s="8" t="s">
+        <v>119</v>
+      </c>
+      <c r="C3" s="8" t="s">
+        <v>120</v>
+      </c>
+      <c r="D3" s="8" t="s">
         <v>121</v>
-      </c>
-      <c r="C3" s="8" t="s">
-        <v>122</v>
-      </c>
-      <c r="D3" s="8" t="s">
-        <v>123</v>
       </c>
     </row>
     <row r="4" ht="45" customHeight="1">
       <c r="A4" s="13" t="s">
+        <v>122</v>
+      </c>
+      <c r="B4" s="13" t="s">
+        <v>123</v>
+      </c>
+      <c r="C4" s="13" t="s">
         <v>124</v>
       </c>
-      <c r="B4" s="13" t="s">
+      <c r="D4" s="13" t="s">
         <v>125</v>
-      </c>
-      <c r="C4" s="13" t="s">
-        <v>126</v>
-      </c>
-      <c r="D4" s="13" t="s">
-        <v>127</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="17" t="s">
-        <v>67</v>
+        <v>71</v>
       </c>
       <c r="B5" s="17" t="n">
         <v>50</v>
@@ -3285,7 +3164,7 @@
         <v>0.001</v>
       </c>
       <c r="D5" s="17" t="s">
-        <v>25</v>
+        <v>29</v>
       </c>
     </row>
     <row r="6">
@@ -3387,44 +3266,44 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="8" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="B3" s="8" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
     </row>
     <row r="4" ht="45" customHeight="1">
       <c r="A4" s="13" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="B4" s="13" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="17" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="B5" s="17" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="17" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="B6" s="17" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
     </row>
     <row r="7">

</xml_diff>